<commit_message>
Update schedule.xlsx from latest solve run
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01984C5X6uigyopTVnDkhSyv
</commit_message>
<xml_diff>
--- a/schedule.xlsx
+++ b/schedule.xlsx
@@ -877,38 +877,38 @@
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>09:15a</t>
         </is>
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>03:00p</t>
         </is>
       </c>
       <c r="M5" s="4" t="n">
-        <v>0</v>
+        <v>5.75</v>
       </c>
       <c r="N5" s="4" t="inlineStr">
         <is>
-          <t>04:45p</t>
+          <t>X</t>
         </is>
       </c>
       <c r="O5" s="4" t="inlineStr">
         <is>
-          <t>10:30p</t>
+          <t>X</t>
         </is>
       </c>
       <c r="P5" s="4" t="n">
-        <v>5.75</v>
+        <v>0</v>
       </c>
       <c r="Q5" s="4" t="inlineStr">
         <is>
-          <t>11:45a</t>
+          <t>10:00a</t>
         </is>
       </c>
       <c r="R5" s="4" t="inlineStr">
         <is>
-          <t>09:45p</t>
+          <t>08:00p</t>
         </is>
       </c>
       <c r="S5" s="4" t="n">
@@ -1055,81 +1055,81 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>10:00a</t>
+          <t>X</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>02:15p</t>
+          <t>X</t>
         </is>
       </c>
       <c r="G7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O7" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R7" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="S7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T7" s="4" t="inlineStr">
+        <is>
+          <t>05:30p</t>
+        </is>
+      </c>
+      <c r="U7" s="4" t="inlineStr">
+        <is>
+          <t>09:45p</t>
+        </is>
+      </c>
+      <c r="V7" s="4" t="n">
         <v>4.25</v>
-      </c>
-      <c r="H7" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I7" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="J7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="L7" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="M7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N7" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="O7" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="P7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q7" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="R7" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="S7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="T7" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="U7" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="V7" s="4" t="n">
-        <v>0</v>
       </c>
       <c r="W7" s="4">
         <f>D7+G7+J7+M7+P7+S7+V7</f>
@@ -1196,16 +1196,16 @@
       </c>
       <c r="N8" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>05:00p</t>
         </is>
       </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>09:15p</t>
         </is>
       </c>
       <c r="P8" s="4" t="n">
-        <v>0</v>
+        <v>4.25</v>
       </c>
       <c r="Q8" s="4" t="inlineStr">
         <is>
@@ -1222,16 +1222,16 @@
       </c>
       <c r="T8" s="4" t="inlineStr">
         <is>
-          <t>05:00p</t>
+          <t>X</t>
         </is>
       </c>
       <c r="U8" s="4" t="inlineStr">
         <is>
-          <t>09:00p</t>
+          <t>X</t>
         </is>
       </c>
       <c r="V8" s="4" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="W8" s="4">
         <f>D8+G8+J8+M8+P8+S8+V8</f>
@@ -1246,25 +1246,25 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>05:30p</t>
+          <t>X</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>09:30p</t>
+          <t>X</t>
         </is>
       </c>
       <c r="D9" s="4" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>05:45p</t>
+          <t>05:15p</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>09:45p</t>
+          <t>09:15p</t>
         </is>
       </c>
       <c r="G9" s="4" t="n">
@@ -1272,29 +1272,29 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>05:00p</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>10:45p</t>
         </is>
       </c>
       <c r="J9" s="4" t="n">
-        <v>0</v>
+        <v>5.75</v>
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>05:30p</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>09:30p</t>
+          <t>X</t>
         </is>
       </c>
       <c r="M9" s="4" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="N9" s="4" t="inlineStr">
         <is>
@@ -1303,11 +1303,11 @@
       </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
-          <t>09:00p</t>
+          <t>10:45p</t>
         </is>
       </c>
       <c r="P9" s="4" t="n">
-        <v>4</v>
+        <v>5.75</v>
       </c>
       <c r="Q9" s="4" t="inlineStr">
         <is>
@@ -1348,16 +1348,16 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>05:45p</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>09:45p</t>
         </is>
       </c>
       <c r="D10" s="4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
@@ -1387,16 +1387,16 @@
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
-          <t>05:00p</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>09:00p</t>
+          <t>X</t>
         </is>
       </c>
       <c r="M10" s="4" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="N10" s="4" t="inlineStr">
         <is>
@@ -1552,16 +1552,16 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>10:00a</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>02:00p</t>
         </is>
       </c>
       <c r="D12" s="4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
@@ -1578,29 +1578,29 @@
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>05:45p</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>10:30p</t>
         </is>
       </c>
       <c r="J12" s="4" t="n">
-        <v>0</v>
+        <v>4.75</v>
       </c>
       <c r="K12" s="4" t="inlineStr">
         <is>
-          <t>11:00a</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L12" s="4" t="inlineStr">
         <is>
-          <t>03:00p</t>
+          <t>X</t>
         </is>
       </c>
       <c r="M12" s="4" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="N12" s="4" t="inlineStr">
         <is>
@@ -1622,24 +1622,24 @@
       </c>
       <c r="R12" s="4" t="inlineStr">
         <is>
-          <t>03:15p</t>
+          <t>03:30p</t>
         </is>
       </c>
       <c r="S12" s="4" t="n">
-        <v>6.25</v>
+        <v>6.5</v>
       </c>
       <c r="T12" s="4" t="inlineStr">
         <is>
-          <t>09:15a</t>
+          <t>05:45p</t>
         </is>
       </c>
       <c r="U12" s="4" t="inlineStr">
         <is>
-          <t>03:00p</t>
+          <t>09:45p</t>
         </is>
       </c>
       <c r="V12" s="4" t="n">
-        <v>5.75</v>
+        <v>4</v>
       </c>
       <c r="W12" s="4">
         <f>D12+G12+J12+M12+P12+S12+V12</f>
@@ -1756,55 +1756,55 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
           <t>05:00p</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>09:00p</t>
         </is>
       </c>
-      <c r="D14" s="4" t="n">
+      <c r="G14" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G14" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="4" t="inlineStr">
+        <is>
           <t>05:00p</t>
         </is>
       </c>
-      <c r="I14" s="4" t="inlineStr">
+      <c r="L14" s="4" t="inlineStr">
         <is>
           <t>09:00p</t>
         </is>
       </c>
-      <c r="J14" s="4" t="n">
+      <c r="M14" s="4" t="n">
         <v>4</v>
-      </c>
-      <c r="K14" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="L14" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="M14" s="4" t="n">
-        <v>0</v>
       </c>
       <c r="N14" s="4" t="inlineStr">
         <is>
@@ -1910,12 +1910,12 @@
       </c>
       <c r="N15" s="4" t="inlineStr">
         <is>
-          <t>12:00p</t>
+          <t>11:00a</t>
         </is>
       </c>
       <c r="O15" s="4" t="inlineStr">
         <is>
-          <t>10:00p</t>
+          <t>09:00p</t>
         </is>
       </c>
       <c r="P15" s="4" t="n">
@@ -1936,7 +1936,7 @@
       </c>
       <c r="T15" s="4" t="inlineStr">
         <is>
-          <t>04:30p</t>
+          <t>04:15p</t>
         </is>
       </c>
       <c r="U15" s="4" t="inlineStr">
@@ -1945,7 +1945,7 @@
         </is>
       </c>
       <c r="V15" s="4" t="n">
-        <v>6.5</v>
+        <v>6.75</v>
       </c>
       <c r="W15" s="4">
         <f>D15+G15+J15+M15+P15+S15+V15</f>
@@ -1960,29 +1960,29 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>11:45a</t>
+          <t>X</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>12:00p</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
           <t>09:45p</t>
         </is>
       </c>
-      <c r="D16" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>11:45a</t>
-        </is>
-      </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>09:45p</t>
-        </is>
-      </c>
       <c r="G16" s="4" t="n">
-        <v>10</v>
+        <v>9.75</v>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
@@ -2004,24 +2004,24 @@
       </c>
       <c r="L16" s="4" t="inlineStr">
         <is>
-          <t>10:45p</t>
+          <t>11:00p</t>
         </is>
       </c>
       <c r="M16" s="4" t="n">
-        <v>6.5</v>
+        <v>6.75</v>
       </c>
       <c r="N16" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>11:15a</t>
         </is>
       </c>
       <c r="O16" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>09:00p</t>
         </is>
       </c>
       <c r="P16" s="4" t="n">
-        <v>0</v>
+        <v>9.75</v>
       </c>
       <c r="Q16" s="4" t="inlineStr">
         <is>
@@ -2038,7 +2038,7 @@
       </c>
       <c r="T16" s="4" t="inlineStr">
         <is>
-          <t>09:15a</t>
+          <t>09:00a</t>
         </is>
       </c>
       <c r="U16" s="4" t="inlineStr">
@@ -2047,7 +2047,7 @@
         </is>
       </c>
       <c r="V16" s="4" t="n">
-        <v>6.75</v>
+        <v>7</v>
       </c>
       <c r="W16" s="4">
         <f>D16+G16+J16+M16+P16+S16+V16</f>
@@ -2127,16 +2127,16 @@
       </c>
       <c r="Q17" s="4" t="inlineStr">
         <is>
-          <t>10:00a</t>
+          <t>05:00p</t>
         </is>
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
-          <t>02:00p</t>
+          <t>09:15p</t>
         </is>
       </c>
       <c r="S17" s="4" t="n">
-        <v>4</v>
+        <v>4.25</v>
       </c>
       <c r="T17" s="4" t="inlineStr">
         <is>
@@ -2190,29 +2190,29 @@
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>05:15p</t>
+          <t>05:00p</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>09:45p</t>
+          <t>09:00p</t>
         </is>
       </c>
       <c r="J18" s="4" t="n">
-        <v>4.5</v>
+        <v>4</v>
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>05:30p</t>
         </is>
       </c>
       <c r="L18" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>09:30p</t>
         </is>
       </c>
       <c r="M18" s="4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N18" s="4" t="inlineStr">
         <is>
@@ -2229,12 +2229,12 @@
       </c>
       <c r="Q18" s="4" t="inlineStr">
         <is>
-          <t>05:30p</t>
+          <t>05:00p</t>
         </is>
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
-          <t>09:30p</t>
+          <t>09:00p</t>
         </is>
       </c>
       <c r="S18" s="4" t="n">
@@ -2242,16 +2242,16 @@
       </c>
       <c r="T18" s="4" t="inlineStr">
         <is>
-          <t>05:30p</t>
+          <t>05:00p</t>
         </is>
       </c>
       <c r="U18" s="4" t="inlineStr">
         <is>
-          <t>09:45p</t>
+          <t>09:00p</t>
         </is>
       </c>
       <c r="V18" s="4" t="n">
-        <v>4.25</v>
+        <v>4</v>
       </c>
       <c r="W18" s="4">
         <f>D18+G18+J18+M18+P18+S18+V18</f>
@@ -2433,16 +2433,16 @@
       </c>
       <c r="Q20" s="4" t="inlineStr">
         <is>
-          <t>05:00p</t>
+          <t>10:00a</t>
         </is>
       </c>
       <c r="R20" s="4" t="inlineStr">
         <is>
-          <t>10:45p</t>
+          <t>02:15p</t>
         </is>
       </c>
       <c r="S20" s="4" t="n">
-        <v>5.75</v>
+        <v>4.25</v>
       </c>
       <c r="T20" s="4" t="inlineStr">
         <is>
@@ -2470,16 +2470,16 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>06:00p</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>10:30p</t>
         </is>
       </c>
       <c r="D21" s="4" t="n">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
@@ -2509,16 +2509,16 @@
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>06:00p</t>
         </is>
       </c>
       <c r="L21" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>10:00p</t>
         </is>
       </c>
       <c r="M21" s="4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N21" s="4" t="inlineStr">
         <is>
@@ -2535,29 +2535,29 @@
       </c>
       <c r="Q21" s="4" t="inlineStr">
         <is>
-          <t>10:00a</t>
+          <t>04:45p</t>
         </is>
       </c>
       <c r="R21" s="4" t="inlineStr">
         <is>
-          <t>02:15p</t>
+          <t>10:30p</t>
         </is>
       </c>
       <c r="S21" s="4" t="n">
-        <v>4.25</v>
+        <v>5.75</v>
       </c>
       <c r="T21" s="4" t="inlineStr">
         <is>
-          <t>10:00a</t>
+          <t>11:00a</t>
         </is>
       </c>
       <c r="U21" s="4" t="inlineStr">
         <is>
-          <t>03:45p</t>
+          <t>03:00p</t>
         </is>
       </c>
       <c r="V21" s="4" t="n">
-        <v>5.75</v>
+        <v>4</v>
       </c>
       <c r="W21" s="4">
         <f>D21+G21+J21+M21+P21+S21+V21</f>
@@ -2598,59 +2598,59 @@
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I22" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N22" s="4" t="inlineStr">
+        <is>
           <t>05:45p</t>
         </is>
       </c>
-      <c r="I22" s="4" t="inlineStr">
-        <is>
-          <t>09:45p</t>
-        </is>
-      </c>
-      <c r="J22" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="K22" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="L22" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="M22" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N22" s="4" t="inlineStr">
-        <is>
-          <t>05:00p</t>
-        </is>
-      </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
-          <t>10:45p</t>
+          <t>10:30p</t>
         </is>
       </c>
       <c r="P22" s="4" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="Q22" s="4" t="inlineStr">
+        <is>
+          <t>04:45p</t>
+        </is>
+      </c>
+      <c r="R22" s="4" t="inlineStr">
+        <is>
+          <t>10:30p</t>
+        </is>
+      </c>
+      <c r="S22" s="4" t="n">
         <v>5.75</v>
       </c>
-      <c r="Q22" s="4" t="inlineStr">
-        <is>
-          <t>04:15p</t>
-        </is>
-      </c>
-      <c r="R22" s="4" t="inlineStr">
-        <is>
-          <t>09:00p</t>
-        </is>
-      </c>
-      <c r="S22" s="4" t="n">
-        <v>4.75</v>
-      </c>
       <c r="T22" s="4" t="inlineStr">
         <is>
-          <t>04:45p</t>
+          <t>06:00p</t>
         </is>
       </c>
       <c r="U22" s="4" t="inlineStr">
@@ -2659,7 +2659,7 @@
         </is>
       </c>
       <c r="V22" s="4" t="n">
-        <v>5.75</v>
+        <v>4.5</v>
       </c>
       <c r="W22" s="4">
         <f>D22+G22+J22+M22+P22+S22+V22</f>
@@ -2674,16 +2674,16 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>05:15p</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>09:15p</t>
         </is>
       </c>
       <c r="D23" s="4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
@@ -2700,16 +2700,16 @@
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>10:45a</t>
+          <t>X</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>03:00p</t>
+          <t>X</t>
         </is>
       </c>
       <c r="J23" s="4" t="n">
-        <v>4.25</v>
+        <v>0</v>
       </c>
       <c r="K23" s="4" t="inlineStr">
         <is>
@@ -2739,7 +2739,7 @@
       </c>
       <c r="Q23" s="4" t="inlineStr">
         <is>
-          <t>06:00p</t>
+          <t>05:45p</t>
         </is>
       </c>
       <c r="R23" s="4" t="inlineStr">
@@ -2748,7 +2748,7 @@
         </is>
       </c>
       <c r="S23" s="4" t="n">
-        <v>4.5</v>
+        <v>4.75</v>
       </c>
       <c r="T23" s="4" t="inlineStr">
         <is>
@@ -2891,16 +2891,16 @@
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>05:00p</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>09:00p</t>
         </is>
       </c>
       <c r="G25" s="4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
@@ -2930,29 +2930,29 @@
       </c>
       <c r="N25" s="4" t="inlineStr">
         <is>
-          <t>05:00p</t>
+          <t>X</t>
         </is>
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
-          <t>09:00p</t>
+          <t>X</t>
         </is>
       </c>
       <c r="P25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q25" s="4" t="inlineStr">
+        <is>
+          <t>10:00a</t>
+        </is>
+      </c>
+      <c r="R25" s="4" t="inlineStr">
+        <is>
+          <t>02:00p</t>
+        </is>
+      </c>
+      <c r="S25" s="4" t="n">
         <v>4</v>
-      </c>
-      <c r="Q25" s="4" t="inlineStr">
-        <is>
-          <t>11:30a</t>
-        </is>
-      </c>
-      <c r="R25" s="4" t="inlineStr">
-        <is>
-          <t>05:15p</t>
-        </is>
-      </c>
-      <c r="S25" s="4" t="n">
-        <v>5.75</v>
       </c>
       <c r="T25" s="4" t="inlineStr">
         <is>
@@ -3134,16 +3134,16 @@
       </c>
       <c r="N27" s="4" t="inlineStr">
         <is>
-          <t>10:00a</t>
+          <t>05:30p</t>
         </is>
       </c>
       <c r="O27" s="4" t="inlineStr">
         <is>
-          <t>02:00p</t>
+          <t>09:45p</t>
         </is>
       </c>
       <c r="P27" s="4" t="n">
-        <v>4</v>
+        <v>4.25</v>
       </c>
       <c r="Q27" s="4" t="inlineStr">
         <is>
@@ -3197,16 +3197,16 @@
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>09:00a</t>
+          <t>09:15a</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>04:00p</t>
+          <t>03:00p</t>
         </is>
       </c>
       <c r="G28" s="4" t="n">
-        <v>7</v>
+        <v>5.75</v>
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
@@ -3215,24 +3215,24 @@
       </c>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>04:00p</t>
+          <t>03:00p</t>
         </is>
       </c>
       <c r="J28" s="4" t="n">
-        <v>6.75</v>
+        <v>5.75</v>
       </c>
       <c r="K28" s="4" t="inlineStr">
         <is>
-          <t>09:00a</t>
+          <t>09:15a</t>
         </is>
       </c>
       <c r="L28" s="4" t="inlineStr">
         <is>
-          <t>03:00p</t>
+          <t>05:00p</t>
         </is>
       </c>
       <c r="M28" s="4" t="n">
-        <v>6</v>
+        <v>7.75</v>
       </c>
       <c r="N28" s="4" t="inlineStr">
         <is>
@@ -3299,55 +3299,55 @@
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>09:15a</t>
+          <t>09:00a</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
+          <t>04:00p</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t>09:00a</t>
+        </is>
+      </c>
+      <c r="I29" s="4" t="inlineStr">
+        <is>
+          <t>05:00p</t>
+        </is>
+      </c>
+      <c r="J29" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="K29" s="4" t="inlineStr">
+        <is>
+          <t>09:00a</t>
+        </is>
+      </c>
+      <c r="L29" s="4" t="inlineStr">
+        <is>
           <t>03:00p</t>
         </is>
       </c>
-      <c r="G29" s="4" t="n">
-        <v>5.75</v>
-      </c>
-      <c r="H29" s="4" t="inlineStr">
-        <is>
-          <t>09:15a</t>
-        </is>
-      </c>
-      <c r="I29" s="4" t="inlineStr">
+      <c r="M29" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="N29" s="4" t="inlineStr">
+        <is>
+          <t>09:00a</t>
+        </is>
+      </c>
+      <c r="O29" s="4" t="inlineStr">
         <is>
           <t>03:00p</t>
         </is>
       </c>
-      <c r="J29" s="4" t="n">
-        <v>5.75</v>
-      </c>
-      <c r="K29" s="4" t="inlineStr">
-        <is>
-          <t>09:15a</t>
-        </is>
-      </c>
-      <c r="L29" s="4" t="inlineStr">
-        <is>
-          <t>05:00p</t>
-        </is>
-      </c>
-      <c r="M29" s="4" t="n">
-        <v>7.75</v>
-      </c>
-      <c r="N29" s="4" t="inlineStr">
-        <is>
-          <t>09:15a</t>
-        </is>
-      </c>
-      <c r="O29" s="4" t="inlineStr">
-        <is>
-          <t>05:00p</t>
-        </is>
-      </c>
       <c r="P29" s="4" t="n">
-        <v>7.75</v>
+        <v>6</v>
       </c>
       <c r="Q29" s="4" t="inlineStr">
         <is>
@@ -3516,42 +3516,42 @@
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I31" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L31" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N31" s="4" t="inlineStr">
+        <is>
           <t>05:00p</t>
         </is>
       </c>
-      <c r="I31" s="4" t="inlineStr">
-        <is>
-          <t>10:45p</t>
-        </is>
-      </c>
-      <c r="J31" s="4" t="n">
-        <v>5.75</v>
-      </c>
-      <c r="K31" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="L31" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="M31" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N31" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>09:00p</t>
         </is>
       </c>
       <c r="P31" s="4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="Q31" s="4" t="inlineStr">
         <is>
@@ -3592,16 +3592,16 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>09:00a</t>
+          <t>09:15a</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>04:00p</t>
+          <t>05:00p</t>
         </is>
       </c>
       <c r="D32" s="4" t="n">
-        <v>7</v>
+        <v>7.75</v>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
@@ -3618,7 +3618,7 @@
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>09:00a</t>
+          <t>09:15a</t>
         </is>
       </c>
       <c r="I32" s="4" t="inlineStr">
@@ -3627,7 +3627,7 @@
         </is>
       </c>
       <c r="J32" s="4" t="n">
-        <v>8</v>
+        <v>7.75</v>
       </c>
       <c r="K32" s="4" t="inlineStr">
         <is>
@@ -3644,7 +3644,7 @@
       </c>
       <c r="N32" s="4" t="inlineStr">
         <is>
-          <t>09:00a</t>
+          <t>09:15a</t>
         </is>
       </c>
       <c r="O32" s="4" t="inlineStr">
@@ -3653,7 +3653,7 @@
         </is>
       </c>
       <c r="P32" s="4" t="n">
-        <v>8</v>
+        <v>7.75</v>
       </c>
       <c r="Q32" s="4" t="inlineStr">
         <is>
@@ -3707,81 +3707,81 @@
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I33" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L33" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N33" s="4" t="inlineStr">
+        <is>
+          <t>05:00p</t>
+        </is>
+      </c>
+      <c r="O33" s="4" t="inlineStr">
+        <is>
+          <t>09:00p</t>
+        </is>
+      </c>
+      <c r="P33" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q33" s="4" t="inlineStr">
+        <is>
+          <t>10:00a</t>
+        </is>
+      </c>
+      <c r="R33" s="4" t="inlineStr">
+        <is>
+          <t>02:15p</t>
+        </is>
+      </c>
+      <c r="S33" s="4" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="T33" s="4" t="inlineStr">
+        <is>
+          <t>10:00a</t>
+        </is>
+      </c>
+      <c r="U33" s="4" t="inlineStr">
+        <is>
           <t>05:15p</t>
         </is>
       </c>
-      <c r="F33" s="4" t="inlineStr">
-        <is>
-          <t>09:15p</t>
-        </is>
-      </c>
-      <c r="G33" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="H33" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I33" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="J33" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K33" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="L33" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="M33" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N33" s="4" t="inlineStr">
-        <is>
-          <t>05:45p</t>
-        </is>
-      </c>
-      <c r="O33" s="4" t="inlineStr">
-        <is>
-          <t>10:30p</t>
-        </is>
-      </c>
-      <c r="P33" s="4" t="n">
-        <v>4.75</v>
-      </c>
-      <c r="Q33" s="4" t="inlineStr">
-        <is>
-          <t>05:45p</t>
-        </is>
-      </c>
-      <c r="R33" s="4" t="inlineStr">
-        <is>
-          <t>10:30p</t>
-        </is>
-      </c>
-      <c r="S33" s="4" t="n">
-        <v>4.75</v>
-      </c>
-      <c r="T33" s="4" t="inlineStr">
-        <is>
-          <t>05:00p</t>
-        </is>
-      </c>
-      <c r="U33" s="4" t="inlineStr">
-        <is>
-          <t>10:45p</t>
-        </is>
-      </c>
       <c r="V33" s="4" t="n">
-        <v>5.75</v>
+        <v>7.25</v>
       </c>
       <c r="W33" s="4">
         <f>D33+G33+J33+M33+P33+S33+V33</f>
@@ -3822,12 +3822,12 @@
       </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t>10:00a</t>
+          <t>10:15a</t>
         </is>
       </c>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>02:00p</t>
+          <t>02:15p</t>
         </is>
       </c>
       <c r="J34" s="4" t="n">
@@ -3950,12 +3950,12 @@
       </c>
       <c r="N35" s="4" t="inlineStr">
         <is>
-          <t>11:00a</t>
+          <t>10:00a</t>
         </is>
       </c>
       <c r="O35" s="4" t="inlineStr">
         <is>
-          <t>03:00p</t>
+          <t>02:00p</t>
         </is>
       </c>
       <c r="P35" s="4" t="n">
@@ -4013,16 +4013,16 @@
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>11:00a</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>03:00p</t>
         </is>
       </c>
       <c r="G36" s="4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H36" s="4" t="inlineStr">
         <is>
@@ -4039,16 +4039,16 @@
       </c>
       <c r="K36" s="4" t="inlineStr">
         <is>
-          <t>10:00a</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>02:00p</t>
+          <t>X</t>
         </is>
       </c>
       <c r="M36" s="4" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
@@ -4102,16 +4102,16 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>04:15p</t>
+          <t>04:30p</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>11:00p</t>
+          <t>10:30p</t>
         </is>
       </c>
       <c r="D37" s="4" t="n">
-        <v>6.75</v>
+        <v>6</v>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
@@ -4141,12 +4141,12 @@
       </c>
       <c r="K37" s="4" t="inlineStr">
         <is>
-          <t>04:15p</t>
+          <t>04:45p</t>
         </is>
       </c>
       <c r="L37" s="4" t="inlineStr">
         <is>
-          <t>10:30p</t>
+          <t>11:00p</t>
         </is>
       </c>
       <c r="M37" s="4" t="n">
@@ -4159,20 +4159,20 @@
       </c>
       <c r="O37" s="4" t="inlineStr">
         <is>
+          <t>10:45p</t>
+        </is>
+      </c>
+      <c r="P37" s="4" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="Q37" s="4" t="inlineStr">
+        <is>
+          <t>12:00p</t>
+        </is>
+      </c>
+      <c r="R37" s="4" t="inlineStr">
+        <is>
           <t>10:00p</t>
-        </is>
-      </c>
-      <c r="P37" s="4" t="n">
-        <v>5.75</v>
-      </c>
-      <c r="Q37" s="4" t="inlineStr">
-        <is>
-          <t>10:00a</t>
-        </is>
-      </c>
-      <c r="R37" s="4" t="inlineStr">
-        <is>
-          <t>08:00p</t>
         </is>
       </c>
       <c r="S37" s="4" t="n">
@@ -4230,16 +4230,16 @@
       </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
-          <t>06:00p</t>
+          <t>05:15p</t>
         </is>
       </c>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>10:30p</t>
+          <t>09:15p</t>
         </is>
       </c>
       <c r="J38" s="4" t="n">
-        <v>4.5</v>
+        <v>4</v>
       </c>
       <c r="K38" s="4" t="inlineStr">
         <is>
@@ -4256,16 +4256,16 @@
       </c>
       <c r="N38" s="4" t="inlineStr">
         <is>
-          <t>04:30p</t>
+          <t>X</t>
         </is>
       </c>
       <c r="O38" s="4" t="inlineStr">
         <is>
-          <t>09:00p</t>
+          <t>X</t>
         </is>
       </c>
       <c r="P38" s="4" t="n">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="Q38" s="4" t="inlineStr">
         <is>
@@ -4282,7 +4282,7 @@
       </c>
       <c r="T38" s="4" t="inlineStr">
         <is>
-          <t>06:00p</t>
+          <t>04:45p</t>
         </is>
       </c>
       <c r="U38" s="4" t="inlineStr">
@@ -4291,7 +4291,7 @@
         </is>
       </c>
       <c r="V38" s="4" t="n">
-        <v>4.5</v>
+        <v>5.75</v>
       </c>
       <c r="W38" s="4">
         <f>D38+G38+J38+M38+P38+S38+V38</f>
@@ -4306,94 +4306,94 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" s="4" t="inlineStr">
+        <is>
           <t>10:00a</t>
         </is>
       </c>
-      <c r="C39" s="4" t="inlineStr">
+      <c r="I39" s="4" t="inlineStr">
         <is>
           <t>02:00p</t>
         </is>
       </c>
-      <c r="D39" s="4" t="n">
+      <c r="J39" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="E39" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F39" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G39" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H39" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I39" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="J39" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="K39" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>10:00a</t>
         </is>
       </c>
       <c r="L39" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>02:00p</t>
         </is>
       </c>
       <c r="M39" s="4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N39" s="4" t="inlineStr">
         <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O39" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P39" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q39" s="4" t="inlineStr">
+        <is>
           <t>06:00p</t>
         </is>
       </c>
-      <c r="O39" s="4" t="inlineStr">
+      <c r="R39" s="4" t="inlineStr">
         <is>
           <t>10:30p</t>
         </is>
       </c>
-      <c r="P39" s="4" t="n">
+      <c r="S39" s="4" t="n">
         <v>4.5</v>
       </c>
-      <c r="Q39" s="4" t="inlineStr">
-        <is>
-          <t>04:45p</t>
-        </is>
-      </c>
-      <c r="R39" s="4" t="inlineStr">
-        <is>
-          <t>10:30p</t>
-        </is>
-      </c>
-      <c r="S39" s="4" t="n">
+      <c r="T39" s="4" t="inlineStr">
+        <is>
+          <t>05:00p</t>
+        </is>
+      </c>
+      <c r="U39" s="4" t="inlineStr">
+        <is>
+          <t>10:45p</t>
+        </is>
+      </c>
+      <c r="V39" s="4" t="n">
         <v>5.75</v>
-      </c>
-      <c r="T39" s="4" t="inlineStr">
-        <is>
-          <t>05:45p</t>
-        </is>
-      </c>
-      <c r="U39" s="4" t="inlineStr">
-        <is>
-          <t>09:45p</t>
-        </is>
-      </c>
-      <c r="V39" s="4" t="n">
-        <v>4</v>
       </c>
       <c r="W39" s="4">
         <f>D39+G39+J39+M39+P39+S39+V39</f>
@@ -4486,16 +4486,16 @@
       </c>
       <c r="T40" s="4" t="inlineStr">
         <is>
-          <t>11:30a</t>
+          <t>10:00a</t>
         </is>
       </c>
       <c r="U40" s="4" t="inlineStr">
         <is>
-          <t>05:15p</t>
+          <t>04:00p</t>
         </is>
       </c>
       <c r="V40" s="4" t="n">
-        <v>5.75</v>
+        <v>6</v>
       </c>
       <c r="W40" s="4">
         <f>D40+G40+J40+M40+P40+S40+V40</f>
@@ -4510,81 +4510,81 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
+          <t>05:30p</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>09:30p</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G41" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" s="4" t="inlineStr">
+        <is>
           <t>06:00p</t>
         </is>
       </c>
-      <c r="C41" s="4" t="inlineStr">
+      <c r="I41" s="4" t="inlineStr">
+        <is>
+          <t>10:15p</t>
+        </is>
+      </c>
+      <c r="J41" s="4" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="K41" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L41" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M41" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N41" s="4" t="inlineStr">
+        <is>
+          <t>06:00p</t>
+        </is>
+      </c>
+      <c r="O41" s="4" t="inlineStr">
         <is>
           <t>10:30p</t>
         </is>
       </c>
-      <c r="D41" s="4" t="n">
+      <c r="P41" s="4" t="n">
         <v>4.5</v>
       </c>
-      <c r="E41" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F41" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G41" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H41" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I41" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="J41" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K41" s="4" t="inlineStr">
-        <is>
-          <t>05:00p</t>
-        </is>
-      </c>
-      <c r="L41" s="4" t="inlineStr">
-        <is>
-          <t>09:15p</t>
-        </is>
-      </c>
-      <c r="M41" s="4" t="n">
-        <v>4.25</v>
-      </c>
-      <c r="N41" s="4" t="inlineStr">
-        <is>
-          <t>05:00p</t>
-        </is>
-      </c>
-      <c r="O41" s="4" t="inlineStr">
-        <is>
-          <t>09:00p</t>
-        </is>
-      </c>
-      <c r="P41" s="4" t="n">
-        <v>4</v>
-      </c>
       <c r="Q41" s="4" t="inlineStr">
         <is>
-          <t>10:00a</t>
+          <t>11:30a</t>
         </is>
       </c>
       <c r="R41" s="4" t="inlineStr">
         <is>
-          <t>02:15p</t>
+          <t>05:15p</t>
         </is>
       </c>
       <c r="S41" s="4" t="n">
-        <v>4.25</v>
+        <v>5.75</v>
       </c>
       <c r="T41" s="4" t="inlineStr">
         <is>
@@ -4714,55 +4714,55 @@
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>09:30a</t>
+          <t>09:00a</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>04:00p</t>
+          <t>03:00p</t>
         </is>
       </c>
       <c r="D43" s="4" t="n">
-        <v>6.5</v>
+        <v>6</v>
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>03:15p</t>
+          <t>02:15p</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>11:00p</t>
+          <t>10:45p</t>
         </is>
       </c>
       <c r="G43" s="4" t="n">
-        <v>7.75</v>
+        <v>8.5</v>
       </c>
       <c r="H43" s="4" t="inlineStr">
         <is>
+          <t>11:45a</t>
+        </is>
+      </c>
+      <c r="I43" s="4" t="inlineStr">
+        <is>
+          <t>09:45p</t>
+        </is>
+      </c>
+      <c r="J43" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="K43" s="4" t="inlineStr">
+        <is>
           <t>12:00p</t>
         </is>
       </c>
-      <c r="I43" s="4" t="inlineStr">
-        <is>
-          <t>09:45p</t>
-        </is>
-      </c>
-      <c r="J43" s="4" t="n">
-        <v>9.75</v>
-      </c>
-      <c r="K43" s="4" t="inlineStr">
-        <is>
-          <t>11:45a</t>
-        </is>
-      </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>09:45p</t>
+          <t>09:30p</t>
         </is>
       </c>
       <c r="M43" s="4" t="n">
-        <v>10</v>
+        <v>9.5</v>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
@@ -4816,7 +4816,7 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>04:45p</t>
+          <t>11:00a</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
@@ -4825,21 +4825,21 @@
         </is>
       </c>
       <c r="D44" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>10:00a</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>02:15p</t>
+        </is>
+      </c>
+      <c r="G44" s="4" t="n">
         <v>4.25</v>
       </c>
-      <c r="E44" s="4" t="inlineStr">
-        <is>
-          <t>11:45a</t>
-        </is>
-      </c>
-      <c r="F44" s="4" t="inlineStr">
-        <is>
-          <t>08:00p</t>
-        </is>
-      </c>
-      <c r="G44" s="4" t="n">
-        <v>8.25</v>
-      </c>
       <c r="H44" s="4" t="inlineStr">
         <is>
           <t>X</t>
@@ -4855,16 +4855,16 @@
       </c>
       <c r="K44" s="4" t="inlineStr">
         <is>
-          <t>09:15a</t>
+          <t>10:15a</t>
         </is>
       </c>
       <c r="L44" s="4" t="inlineStr">
         <is>
-          <t>03:00p</t>
+          <t>02:15p</t>
         </is>
       </c>
       <c r="M44" s="4" t="n">
-        <v>5.75</v>
+        <v>4</v>
       </c>
       <c r="N44" s="4" t="inlineStr">
         <is>
@@ -5148,25 +5148,25 @@
         </is>
       </c>
       <c r="B54" s="5" t="n">
-        <v>108.25</v>
+        <v>107.5</v>
       </c>
       <c r="E54" s="5" t="n">
-        <v>103.5</v>
+        <v>104.25</v>
       </c>
       <c r="H54" s="5" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K54" s="5" t="n">
-        <v>107.5</v>
+        <v>107</v>
       </c>
       <c r="N54" s="5" t="n">
-        <v>122.75</v>
+        <v>121.5</v>
       </c>
       <c r="Q54" s="5" t="n">
-        <v>105.5</v>
+        <v>105.25</v>
       </c>
       <c r="T54" s="5" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="W54" s="5">
         <f>SUM(B54:T54)</f>
@@ -5328,7 +5328,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>+9.8</t>
+          <t>+9.0</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -5347,13 +5347,13 @@
         <v>8</v>
       </c>
       <c r="H60" t="n">
+        <v>7</v>
+      </c>
+      <c r="I60" t="n">
+        <v>6</v>
+      </c>
+      <c r="J60" t="n">
         <v>8</v>
-      </c>
-      <c r="I60" t="n">
-        <v>5</v>
-      </c>
-      <c r="J60" t="n">
-        <v>7</v>
       </c>
       <c r="K60" t="n">
         <v>6</v>
@@ -5370,7 +5370,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>+8.0</t>
+          <t>+8.8</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -5392,13 +5392,13 @@
         <v>7</v>
       </c>
       <c r="I61" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J61" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K61" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L61" t="n">
         <v>6</v>
@@ -5412,7 +5412,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>-3.0</t>
+          <t>-2.0</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -5434,16 +5434,16 @@
         <v>8</v>
       </c>
       <c r="I62" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J62" t="n">
         <v>8</v>
       </c>
       <c r="K62" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L62" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="63">
@@ -5454,7 +5454,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>+3.5</t>
+          <t>+3.0</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -5496,7 +5496,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>+9.8</t>
+          <t>+8.5</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -5524,7 +5524,7 @@
         <v>8</v>
       </c>
       <c r="K64" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L64" t="n">
         <v>6</v>
@@ -5538,7 +5538,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>-2.5</t>
+          <t>-2.8</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -5580,7 +5580,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>+4.5</t>
+          <t>+5.5</t>
         </is>
       </c>
       <c r="C66" t="n">

</xml_diff>

<commit_message>
Update schedule.xlsx from solve with corrected Sunday targets
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01984C5X6uigyopTVnDkhSyv
</commit_message>
<xml_diff>
--- a/schedule.xlsx
+++ b/schedule.xlsx
@@ -673,7 +673,7 @@
       </c>
       <c r="K3" s="4" t="inlineStr">
         <is>
-          <t>02:15p</t>
+          <t>02:00p</t>
         </is>
       </c>
       <c r="L3" s="4" t="inlineStr">
@@ -682,7 +682,7 @@
         </is>
       </c>
       <c r="M3" s="4" t="n">
-        <v>8.75</v>
+        <v>9</v>
       </c>
       <c r="N3" s="4" t="inlineStr">
         <is>
@@ -814,16 +814,16 @@
       </c>
       <c r="T4" s="4" t="inlineStr">
         <is>
-          <t>11:00a</t>
+          <t>11:30a</t>
         </is>
       </c>
       <c r="U4" s="4" t="inlineStr">
         <is>
-          <t>03:00p</t>
+          <t>05:15p</t>
         </is>
       </c>
       <c r="V4" s="4" t="n">
-        <v>4</v>
+        <v>5.75</v>
       </c>
       <c r="W4" s="4">
         <f>D4+G4+J4+M4+P4+S4+V4</f>
@@ -843,72 +843,72 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
+          <t>10:45p</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>05:00p</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>11:00p</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" s="4" t="inlineStr">
+        <is>
+          <t>04:45p</t>
+        </is>
+      </c>
+      <c r="O5" s="4" t="inlineStr">
+        <is>
           <t>10:30p</t>
         </is>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="P5" s="4" t="n">
         <v>5.75</v>
       </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>05:00p</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>10:45p</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="n">
-        <v>5.75</v>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I5" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="J5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" s="4" t="inlineStr">
-        <is>
-          <t>09:15a</t>
-        </is>
-      </c>
-      <c r="L5" s="4" t="inlineStr">
-        <is>
-          <t>03:00p</t>
-        </is>
-      </c>
-      <c r="M5" s="4" t="n">
-        <v>5.75</v>
-      </c>
-      <c r="N5" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="O5" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="P5" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="Q5" s="4" t="inlineStr">
         <is>
-          <t>10:00a</t>
+          <t>11:45a</t>
         </is>
       </c>
       <c r="R5" s="4" t="inlineStr">
         <is>
-          <t>08:00p</t>
+          <t>09:45p</t>
         </is>
       </c>
       <c r="S5" s="4" t="n">
@@ -921,11 +921,11 @@
       </c>
       <c r="U5" s="4" t="inlineStr">
         <is>
-          <t>05:45p</t>
+          <t>05:15p</t>
         </is>
       </c>
       <c r="V5" s="4" t="n">
-        <v>7.75</v>
+        <v>7.25</v>
       </c>
       <c r="W5" s="4">
         <f>D5+G5+J5+M5+P5+S5+V5</f>
@@ -1068,16 +1068,16 @@
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>05:00p</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>09:15p</t>
         </is>
       </c>
       <c r="J7" s="4" t="n">
-        <v>0</v>
+        <v>4.25</v>
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
@@ -1120,16 +1120,16 @@
       </c>
       <c r="T7" s="4" t="inlineStr">
         <is>
-          <t>05:30p</t>
+          <t>X</t>
         </is>
       </c>
       <c r="U7" s="4" t="inlineStr">
         <is>
-          <t>09:45p</t>
+          <t>X</t>
         </is>
       </c>
       <c r="V7" s="4" t="n">
-        <v>4.25</v>
+        <v>0</v>
       </c>
       <c r="W7" s="4">
         <f>D7+G7+J7+M7+P7+S7+V7</f>
@@ -1196,16 +1196,16 @@
       </c>
       <c r="N8" s="4" t="inlineStr">
         <is>
-          <t>05:00p</t>
+          <t>X</t>
         </is>
       </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
-          <t>09:15p</t>
+          <t>X</t>
         </is>
       </c>
       <c r="P8" s="4" t="n">
-        <v>4.25</v>
+        <v>0</v>
       </c>
       <c r="Q8" s="4" t="inlineStr">
         <is>
@@ -1222,16 +1222,16 @@
       </c>
       <c r="T8" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>06:00p</t>
         </is>
       </c>
       <c r="U8" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>10:30p</t>
         </is>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="W8" s="4">
         <f>D8+G8+J8+M8+P8+S8+V8</f>
@@ -1246,68 +1246,68 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>05:45p</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>09:45p</t>
         </is>
       </c>
       <c r="D9" s="4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>05:00p</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>09:00p</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t>05:00p</t>
+        </is>
+      </c>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t>09:00p</t>
+        </is>
+      </c>
+      <c r="M9" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="N9" s="4" t="inlineStr">
+        <is>
           <t>05:15p</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="O9" s="4" t="inlineStr">
         <is>
           <t>09:15p</t>
         </is>
       </c>
-      <c r="G9" s="4" t="n">
+      <c r="P9" s="4" t="n">
         <v>4</v>
-      </c>
-      <c r="H9" s="4" t="inlineStr">
-        <is>
-          <t>05:00p</t>
-        </is>
-      </c>
-      <c r="I9" s="4" t="inlineStr">
-        <is>
-          <t>10:45p</t>
-        </is>
-      </c>
-      <c r="J9" s="4" t="n">
-        <v>5.75</v>
-      </c>
-      <c r="K9" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="L9" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="M9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N9" s="4" t="inlineStr">
-        <is>
-          <t>05:00p</t>
-        </is>
-      </c>
-      <c r="O9" s="4" t="inlineStr">
-        <is>
-          <t>10:45p</t>
-        </is>
-      </c>
-      <c r="P9" s="4" t="n">
-        <v>5.75</v>
       </c>
       <c r="Q9" s="4" t="inlineStr">
         <is>
@@ -1348,55 +1348,55 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>05:45p</t>
+          <t>X</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>09:45p</t>
+          <t>X</t>
         </is>
       </c>
       <c r="D10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="4" t="inlineStr">
+        <is>
+          <t>05:00p</t>
+        </is>
+      </c>
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t>09:00p</t>
+        </is>
+      </c>
+      <c r="M10" s="4" t="n">
         <v>4</v>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I10" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="J10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="L10" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="M10" s="4" t="n">
-        <v>0</v>
       </c>
       <c r="N10" s="4" t="inlineStr">
         <is>
@@ -1552,94 +1552,94 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>10:00a</t>
+          <t>X</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>02:00p</t>
+          <t>X</t>
         </is>
       </c>
       <c r="D12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>11:00a</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>03:00p</t>
+        </is>
+      </c>
+      <c r="J12" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F12" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H12" s="4" t="inlineStr">
-        <is>
-          <t>05:45p</t>
-        </is>
-      </c>
-      <c r="I12" s="4" t="inlineStr">
-        <is>
-          <t>10:30p</t>
-        </is>
-      </c>
-      <c r="J12" s="4" t="n">
-        <v>4.75</v>
-      </c>
       <c r="K12" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>05:30p</t>
         </is>
       </c>
       <c r="L12" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>09:30p</t>
         </is>
       </c>
       <c r="M12" s="4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N12" s="4" t="inlineStr">
         <is>
-          <t>11:00a</t>
+          <t>X</t>
         </is>
       </c>
       <c r="O12" s="4" t="inlineStr">
         <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="4" t="inlineStr">
+        <is>
+          <t>09:00a</t>
+        </is>
+      </c>
+      <c r="R12" s="4" t="inlineStr">
+        <is>
+          <t>03:15p</t>
+        </is>
+      </c>
+      <c r="S12" s="4" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="T12" s="4" t="inlineStr">
+        <is>
+          <t>09:15a</t>
+        </is>
+      </c>
+      <c r="U12" s="4" t="inlineStr">
+        <is>
           <t>03:00p</t>
         </is>
       </c>
-      <c r="P12" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q12" s="4" t="inlineStr">
-        <is>
-          <t>09:00a</t>
-        </is>
-      </c>
-      <c r="R12" s="4" t="inlineStr">
-        <is>
-          <t>03:30p</t>
-        </is>
-      </c>
-      <c r="S12" s="4" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="T12" s="4" t="inlineStr">
-        <is>
-          <t>05:45p</t>
-        </is>
-      </c>
-      <c r="U12" s="4" t="inlineStr">
-        <is>
-          <t>09:45p</t>
-        </is>
-      </c>
       <c r="V12" s="4" t="n">
-        <v>4</v>
+        <v>5.75</v>
       </c>
       <c r="W12" s="4">
         <f>D12+G12+J12+M12+P12+S12+V12</f>
@@ -1769,29 +1769,29 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
           <t>05:00p</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>09:00p</t>
         </is>
       </c>
-      <c r="G14" s="4" t="n">
+      <c r="J14" s="4" t="n">
         <v>4</v>
-      </c>
-      <c r="H14" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I14" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="J14" s="4" t="n">
-        <v>0</v>
       </c>
       <c r="K14" s="4" t="inlineStr">
         <is>
@@ -1834,12 +1834,12 @@
       </c>
       <c r="T14" s="4" t="inlineStr">
         <is>
-          <t>11:30a</t>
+          <t>11:00a</t>
         </is>
       </c>
       <c r="U14" s="4" t="inlineStr">
         <is>
-          <t>03:30p</t>
+          <t>03:00p</t>
         </is>
       </c>
       <c r="V14" s="4" t="n">
@@ -1876,11 +1876,11 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>10:15p</t>
+          <t>10:00p</t>
         </is>
       </c>
       <c r="G15" s="4" t="n">
-        <v>6</v>
+        <v>5.75</v>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
@@ -1960,20 +1960,20 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>11:45a</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>09:15p</t>
         </is>
       </c>
       <c r="D16" s="4" t="n">
-        <v>0</v>
+        <v>9.5</v>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>12:00p</t>
+          <t>11:45a</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
@@ -1982,7 +1982,7 @@
         </is>
       </c>
       <c r="G16" s="4" t="n">
-        <v>9.75</v>
+        <v>10</v>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
@@ -2012,16 +2012,16 @@
       </c>
       <c r="N16" s="4" t="inlineStr">
         <is>
-          <t>11:15a</t>
+          <t>X</t>
         </is>
       </c>
       <c r="O16" s="4" t="inlineStr">
         <is>
-          <t>09:00p</t>
+          <t>X</t>
         </is>
       </c>
       <c r="P16" s="4" t="n">
-        <v>9.75</v>
+        <v>0</v>
       </c>
       <c r="Q16" s="4" t="inlineStr">
         <is>
@@ -2132,11 +2132,11 @@
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
-          <t>09:15p</t>
+          <t>10:45p</t>
         </is>
       </c>
       <c r="S17" s="4" t="n">
-        <v>4.25</v>
+        <v>5.75</v>
       </c>
       <c r="T17" s="4" t="inlineStr">
         <is>
@@ -2190,29 +2190,29 @@
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>05:00p</t>
+          <t>05:30p</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>09:00p</t>
+          <t>09:45p</t>
         </is>
       </c>
       <c r="J18" s="4" t="n">
-        <v>4</v>
+        <v>4.25</v>
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>05:30p</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L18" s="4" t="inlineStr">
         <is>
-          <t>09:30p</t>
+          <t>X</t>
         </is>
       </c>
       <c r="M18" s="4" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="N18" s="4" t="inlineStr">
         <is>
@@ -2433,16 +2433,16 @@
       </c>
       <c r="Q20" s="4" t="inlineStr">
         <is>
-          <t>10:00a</t>
+          <t>05:00p</t>
         </is>
       </c>
       <c r="R20" s="4" t="inlineStr">
         <is>
-          <t>02:15p</t>
+          <t>10:45p</t>
         </is>
       </c>
       <c r="S20" s="4" t="n">
-        <v>4.25</v>
+        <v>5.75</v>
       </c>
       <c r="T20" s="4" t="inlineStr">
         <is>
@@ -2470,81 +2470,81 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>06:00p</t>
+          <t>X</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I21" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O21" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q21" s="4" t="inlineStr">
+        <is>
+          <t>05:45p</t>
+        </is>
+      </c>
+      <c r="R21" s="4" t="inlineStr">
+        <is>
           <t>10:30p</t>
         </is>
       </c>
-      <c r="D21" s="4" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G21" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H21" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I21" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="J21" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K21" s="4" t="inlineStr">
-        <is>
-          <t>06:00p</t>
-        </is>
-      </c>
-      <c r="L21" s="4" t="inlineStr">
-        <is>
-          <t>10:00p</t>
-        </is>
-      </c>
-      <c r="M21" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="N21" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="O21" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="P21" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q21" s="4" t="inlineStr">
-        <is>
-          <t>04:45p</t>
-        </is>
-      </c>
-      <c r="R21" s="4" t="inlineStr">
-        <is>
-          <t>10:30p</t>
-        </is>
-      </c>
       <c r="S21" s="4" t="n">
-        <v>5.75</v>
+        <v>4.75</v>
       </c>
       <c r="T21" s="4" t="inlineStr">
         <is>
@@ -2650,7 +2650,7 @@
       </c>
       <c r="T22" s="4" t="inlineStr">
         <is>
-          <t>06:00p</t>
+          <t>04:45p</t>
         </is>
       </c>
       <c r="U22" s="4" t="inlineStr">
@@ -2659,7 +2659,7 @@
         </is>
       </c>
       <c r="V22" s="4" t="n">
-        <v>4.5</v>
+        <v>5.75</v>
       </c>
       <c r="W22" s="4">
         <f>D22+G22+J22+M22+P22+S22+V22</f>
@@ -2674,30 +2674,30 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>05:15p</t>
+          <t>X</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>09:15p</t>
+          <t>X</t>
         </is>
       </c>
       <c r="D23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>10:00a</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>02:00p</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F23" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G23" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
           <t>X</t>
@@ -2739,29 +2739,29 @@
       </c>
       <c r="Q23" s="4" t="inlineStr">
         <is>
+          <t>10:00a</t>
+        </is>
+      </c>
+      <c r="R23" s="4" t="inlineStr">
+        <is>
+          <t>02:15p</t>
+        </is>
+      </c>
+      <c r="S23" s="4" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="T23" s="4" t="inlineStr">
+        <is>
           <t>05:45p</t>
         </is>
       </c>
-      <c r="R23" s="4" t="inlineStr">
+      <c r="U23" s="4" t="inlineStr">
         <is>
           <t>10:30p</t>
         </is>
       </c>
-      <c r="S23" s="4" t="n">
+      <c r="V23" s="4" t="n">
         <v>4.75</v>
-      </c>
-      <c r="T23" s="4" t="inlineStr">
-        <is>
-          <t>11:00a</t>
-        </is>
-      </c>
-      <c r="U23" s="4" t="inlineStr">
-        <is>
-          <t>03:00p</t>
-        </is>
-      </c>
-      <c r="V23" s="4" t="n">
-        <v>4</v>
       </c>
       <c r="W23" s="4">
         <f>D23+G23+J23+M23+P23+S23+V23</f>
@@ -2789,29 +2789,29 @@
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
           <t>10:00a</t>
         </is>
       </c>
-      <c r="F24" s="4" t="inlineStr">
+      <c r="I24" s="4" t="inlineStr">
         <is>
           <t>02:00p</t>
         </is>
       </c>
-      <c r="G24" s="4" t="n">
+      <c r="J24" s="4" t="n">
         <v>4</v>
-      </c>
-      <c r="H24" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I24" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="J24" s="4" t="n">
-        <v>0</v>
       </c>
       <c r="K24" s="4" t="inlineStr">
         <is>
@@ -2878,69 +2878,69 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>05:00p</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>09:00p</t>
         </is>
       </c>
       <c r="D25" s="4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I25" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N25" s="4" t="inlineStr">
+        <is>
           <t>05:00p</t>
         </is>
       </c>
-      <c r="F25" s="4" t="inlineStr">
+      <c r="O25" s="4" t="inlineStr">
         <is>
           <t>09:00p</t>
         </is>
       </c>
-      <c r="G25" s="4" t="n">
+      <c r="P25" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="H25" s="4" t="inlineStr">
-        <is>
-          <t>05:00p</t>
-        </is>
-      </c>
-      <c r="I25" s="4" t="inlineStr">
-        <is>
-          <t>09:00p</t>
-        </is>
-      </c>
-      <c r="J25" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="K25" s="4" t="inlineStr">
-        <is>
-          <t>05:00p</t>
-        </is>
-      </c>
-      <c r="L25" s="4" t="inlineStr">
-        <is>
-          <t>09:00p</t>
-        </is>
-      </c>
-      <c r="M25" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="N25" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="O25" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="P25" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="Q25" s="4" t="inlineStr">
         <is>
           <t>10:00a</t>
@@ -2948,11 +2948,11 @@
       </c>
       <c r="R25" s="4" t="inlineStr">
         <is>
-          <t>02:00p</t>
+          <t>05:15p</t>
         </is>
       </c>
       <c r="S25" s="4" t="n">
-        <v>4</v>
+        <v>7.25</v>
       </c>
       <c r="T25" s="4" t="inlineStr">
         <is>
@@ -3134,16 +3134,16 @@
       </c>
       <c r="N27" s="4" t="inlineStr">
         <is>
-          <t>05:30p</t>
+          <t>10:00a</t>
         </is>
       </c>
       <c r="O27" s="4" t="inlineStr">
         <is>
-          <t>09:45p</t>
+          <t>02:00p</t>
         </is>
       </c>
       <c r="P27" s="4" t="n">
-        <v>4.25</v>
+        <v>4</v>
       </c>
       <c r="Q27" s="4" t="inlineStr">
         <is>
@@ -3189,41 +3189,41 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
+          <t>03:00p</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>09:00a</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>03:00p</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>09:15a</t>
+        </is>
+      </c>
+      <c r="I28" s="4" t="inlineStr">
+        <is>
           <t>05:00p</t>
         </is>
       </c>
-      <c r="D28" s="4" t="n">
+      <c r="J28" s="4" t="n">
         <v>7.75</v>
       </c>
-      <c r="E28" s="4" t="inlineStr">
-        <is>
-          <t>09:15a</t>
-        </is>
-      </c>
-      <c r="F28" s="4" t="inlineStr">
-        <is>
-          <t>03:00p</t>
-        </is>
-      </c>
-      <c r="G28" s="4" t="n">
-        <v>5.75</v>
-      </c>
-      <c r="H28" s="4" t="inlineStr">
-        <is>
-          <t>09:15a</t>
-        </is>
-      </c>
-      <c r="I28" s="4" t="inlineStr">
-        <is>
-          <t>03:00p</t>
-        </is>
-      </c>
-      <c r="J28" s="4" t="n">
-        <v>5.75</v>
-      </c>
       <c r="K28" s="4" t="inlineStr">
         <is>
-          <t>09:15a</t>
+          <t>09:00a</t>
         </is>
       </c>
       <c r="L28" s="4" t="inlineStr">
@@ -3232,7 +3232,7 @@
         </is>
       </c>
       <c r="M28" s="4" t="n">
-        <v>7.75</v>
+        <v>8</v>
       </c>
       <c r="N28" s="4" t="inlineStr">
         <is>
@@ -3317,11 +3317,11 @@
       </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>05:00p</t>
+          <t>03:00p</t>
         </is>
       </c>
       <c r="J29" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="K29" s="4" t="inlineStr">
         <is>
@@ -3343,11 +3343,11 @@
       </c>
       <c r="O29" s="4" t="inlineStr">
         <is>
-          <t>03:00p</t>
+          <t>05:00p</t>
         </is>
       </c>
       <c r="P29" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="Q29" s="4" t="inlineStr">
         <is>
@@ -3542,16 +3542,16 @@
       </c>
       <c r="N31" s="4" t="inlineStr">
         <is>
-          <t>05:00p</t>
+          <t>06:00p</t>
         </is>
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
-          <t>09:00p</t>
+          <t>10:30p</t>
         </is>
       </c>
       <c r="P31" s="4" t="n">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="Q31" s="4" t="inlineStr">
         <is>
@@ -3592,29 +3592,29 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
+          <t>09:00a</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>05:00p</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
           <t>09:15a</t>
         </is>
       </c>
-      <c r="C32" s="4" t="inlineStr">
-        <is>
-          <t>05:00p</t>
-        </is>
-      </c>
-      <c r="D32" s="4" t="n">
-        <v>7.75</v>
-      </c>
-      <c r="E32" s="4" t="inlineStr">
-        <is>
-          <t>09:00a</t>
-        </is>
-      </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
           <t>03:00p</t>
         </is>
       </c>
       <c r="G32" s="4" t="n">
-        <v>6</v>
+        <v>5.75</v>
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
@@ -3631,7 +3631,7 @@
       </c>
       <c r="K32" s="4" t="inlineStr">
         <is>
-          <t>09:00a</t>
+          <t>09:15a</t>
         </is>
       </c>
       <c r="L32" s="4" t="inlineStr">
@@ -3640,7 +3640,7 @@
         </is>
       </c>
       <c r="M32" s="4" t="n">
-        <v>6</v>
+        <v>5.75</v>
       </c>
       <c r="N32" s="4" t="inlineStr">
         <is>
@@ -3707,16 +3707,16 @@
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>06:00p</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>10:00p</t>
         </is>
       </c>
       <c r="G33" s="4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
@@ -3759,29 +3759,29 @@
       </c>
       <c r="Q33" s="4" t="inlineStr">
         <is>
-          <t>10:00a</t>
+          <t>05:00p</t>
         </is>
       </c>
       <c r="R33" s="4" t="inlineStr">
         <is>
-          <t>02:15p</t>
+          <t>09:00p</t>
         </is>
       </c>
       <c r="S33" s="4" t="n">
-        <v>4.25</v>
+        <v>4</v>
       </c>
       <c r="T33" s="4" t="inlineStr">
         <is>
-          <t>10:00a</t>
+          <t>05:00p</t>
         </is>
       </c>
       <c r="U33" s="4" t="inlineStr">
         <is>
-          <t>05:15p</t>
+          <t>10:45p</t>
         </is>
       </c>
       <c r="V33" s="4" t="n">
-        <v>7.25</v>
+        <v>5.75</v>
       </c>
       <c r="W33" s="4">
         <f>D33+G33+J33+M33+P33+S33+V33</f>
@@ -3796,16 +3796,16 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>05:30p</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>09:30p</t>
         </is>
       </c>
       <c r="D34" s="4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
@@ -3822,16 +3822,16 @@
       </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t>10:15a</t>
+          <t>X</t>
         </is>
       </c>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>02:15p</t>
+          <t>X</t>
         </is>
       </c>
       <c r="J34" s="4" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K34" s="4" t="inlineStr">
         <is>
@@ -4013,12 +4013,12 @@
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>11:00a</t>
+          <t>10:00a</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>03:00p</t>
+          <t>02:00p</t>
         </is>
       </c>
       <c r="G36" s="4" t="n">
@@ -4039,29 +4039,29 @@
       </c>
       <c r="K36" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>11:00a</t>
         </is>
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>03:00p</t>
         </is>
       </c>
       <c r="M36" s="4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>11:00a</t>
         </is>
       </c>
       <c r="O36" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>03:00p</t>
         </is>
       </c>
       <c r="P36" s="4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="Q36" s="4" t="inlineStr">
         <is>
@@ -4102,68 +4102,68 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>04:30p</t>
+          <t>04:15p</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>10:30p</t>
+          <t>11:00p</t>
         </is>
       </c>
       <c r="D37" s="4" t="n">
-        <v>6</v>
+        <v>6.75</v>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>04:30p</t>
+          <t>05:00p</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
+          <t>10:45p</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="H37" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I37" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K37" s="4" t="inlineStr">
+        <is>
+          <t>04:15p</t>
+        </is>
+      </c>
+      <c r="L37" s="4" t="inlineStr">
+        <is>
           <t>11:00p</t>
         </is>
       </c>
-      <c r="G37" s="4" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="H37" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I37" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="J37" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K37" s="4" t="inlineStr">
-        <is>
-          <t>04:45p</t>
-        </is>
-      </c>
-      <c r="L37" s="4" t="inlineStr">
+      <c r="M37" s="4" t="n">
+        <v>6.75</v>
+      </c>
+      <c r="N37" s="4" t="inlineStr">
+        <is>
+          <t>04:15p</t>
+        </is>
+      </c>
+      <c r="O37" s="4" t="inlineStr">
         <is>
           <t>11:00p</t>
         </is>
       </c>
-      <c r="M37" s="4" t="n">
-        <v>6.25</v>
-      </c>
-      <c r="N37" s="4" t="inlineStr">
-        <is>
-          <t>04:15p</t>
-        </is>
-      </c>
-      <c r="O37" s="4" t="inlineStr">
-        <is>
-          <t>10:45p</t>
-        </is>
-      </c>
       <c r="P37" s="4" t="n">
-        <v>6.5</v>
+        <v>6.75</v>
       </c>
       <c r="Q37" s="4" t="inlineStr">
         <is>
@@ -4230,16 +4230,16 @@
       </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
-          <t>05:15p</t>
+          <t>05:45p</t>
         </is>
       </c>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>09:15p</t>
+          <t>10:30p</t>
         </is>
       </c>
       <c r="J38" s="4" t="n">
-        <v>4</v>
+        <v>4.75</v>
       </c>
       <c r="K38" s="4" t="inlineStr">
         <is>
@@ -4256,20 +4256,20 @@
       </c>
       <c r="N38" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>05:30p</t>
         </is>
       </c>
       <c r="O38" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>09:45p</t>
         </is>
       </c>
       <c r="P38" s="4" t="n">
-        <v>0</v>
+        <v>4.25</v>
       </c>
       <c r="Q38" s="4" t="inlineStr">
         <is>
-          <t>04:45p</t>
+          <t>06:00p</t>
         </is>
       </c>
       <c r="R38" s="4" t="inlineStr">
@@ -4278,20 +4278,20 @@
         </is>
       </c>
       <c r="S38" s="4" t="n">
-        <v>5.75</v>
+        <v>4.5</v>
       </c>
       <c r="T38" s="4" t="inlineStr">
         <is>
-          <t>04:45p</t>
+          <t>05:30p</t>
         </is>
       </c>
       <c r="U38" s="4" t="inlineStr">
         <is>
-          <t>10:30p</t>
+          <t>09:45p</t>
         </is>
       </c>
       <c r="V38" s="4" t="n">
-        <v>5.75</v>
+        <v>4.25</v>
       </c>
       <c r="W38" s="4">
         <f>D38+G38+J38+M38+P38+S38+V38</f>
@@ -4332,16 +4332,16 @@
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>10:00a</t>
+          <t>X</t>
         </is>
       </c>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>02:00p</t>
+          <t>X</t>
         </is>
       </c>
       <c r="J39" s="4" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K39" s="4" t="inlineStr">
         <is>
@@ -4358,42 +4358,42 @@
       </c>
       <c r="N39" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>05:00p</t>
         </is>
       </c>
       <c r="O39" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>09:00p</t>
         </is>
       </c>
       <c r="P39" s="4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="Q39" s="4" t="inlineStr">
         <is>
-          <t>06:00p</t>
+          <t>10:00a</t>
         </is>
       </c>
       <c r="R39" s="4" t="inlineStr">
         <is>
-          <t>10:30p</t>
+          <t>02:00p</t>
         </is>
       </c>
       <c r="S39" s="4" t="n">
-        <v>4.5</v>
+        <v>4</v>
       </c>
       <c r="T39" s="4" t="inlineStr">
         <is>
-          <t>05:00p</t>
+          <t>11:00a</t>
         </is>
       </c>
       <c r="U39" s="4" t="inlineStr">
         <is>
-          <t>10:45p</t>
+          <t>03:00p</t>
         </is>
       </c>
       <c r="V39" s="4" t="n">
-        <v>5.75</v>
+        <v>4</v>
       </c>
       <c r="W39" s="4">
         <f>D39+G39+J39+M39+P39+S39+V39</f>
@@ -4460,12 +4460,12 @@
       </c>
       <c r="N40" s="4" t="inlineStr">
         <is>
-          <t>10:00a</t>
+          <t>11:00a</t>
         </is>
       </c>
       <c r="O40" s="4" t="inlineStr">
         <is>
-          <t>02:00p</t>
+          <t>03:00p</t>
         </is>
       </c>
       <c r="P40" s="4" t="n">
@@ -4491,11 +4491,11 @@
       </c>
       <c r="U40" s="4" t="inlineStr">
         <is>
-          <t>04:00p</t>
+          <t>03:45p</t>
         </is>
       </c>
       <c r="V40" s="4" t="n">
-        <v>6</v>
+        <v>5.75</v>
       </c>
       <c r="W40" s="4">
         <f>D40+G40+J40+M40+P40+S40+V40</f>
@@ -4510,30 +4510,30 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
+          <t>06:00p</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>10:30p</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
           <t>05:30p</t>
         </is>
       </c>
-      <c r="C41" s="4" t="inlineStr">
+      <c r="F41" s="4" t="inlineStr">
         <is>
           <t>09:30p</t>
         </is>
       </c>
-      <c r="D41" s="4" t="n">
+      <c r="G41" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="E41" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F41" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G41" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
           <t>06:00p</t>
@@ -4541,50 +4541,50 @@
       </c>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>10:15p</t>
+          <t>10:30p</t>
         </is>
       </c>
       <c r="J41" s="4" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="K41" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L41" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M41" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N41" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O41" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P41" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q41" s="4" t="inlineStr">
+        <is>
+          <t>10:00a</t>
+        </is>
+      </c>
+      <c r="R41" s="4" t="inlineStr">
+        <is>
+          <t>02:15p</t>
+        </is>
+      </c>
+      <c r="S41" s="4" t="n">
         <v>4.25</v>
-      </c>
-      <c r="K41" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="L41" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="M41" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N41" s="4" t="inlineStr">
-        <is>
-          <t>06:00p</t>
-        </is>
-      </c>
-      <c r="O41" s="4" t="inlineStr">
-        <is>
-          <t>10:30p</t>
-        </is>
-      </c>
-      <c r="P41" s="4" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="Q41" s="4" t="inlineStr">
-        <is>
-          <t>11:30a</t>
-        </is>
-      </c>
-      <c r="R41" s="4" t="inlineStr">
-        <is>
-          <t>05:15p</t>
-        </is>
-      </c>
-      <c r="S41" s="4" t="n">
-        <v>5.75</v>
       </c>
       <c r="T41" s="4" t="inlineStr">
         <is>
@@ -4714,7 +4714,7 @@
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>09:00a</t>
+          <t>09:15a</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
@@ -4723,11 +4723,11 @@
         </is>
       </c>
       <c r="D43" s="4" t="n">
-        <v>6</v>
+        <v>5.75</v>
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>02:15p</t>
+          <t>02:00p</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
@@ -4736,7 +4736,7 @@
         </is>
       </c>
       <c r="G43" s="4" t="n">
-        <v>8.5</v>
+        <v>8.75</v>
       </c>
       <c r="H43" s="4" t="inlineStr">
         <is>
@@ -4745,24 +4745,24 @@
       </c>
       <c r="I43" s="4" t="inlineStr">
         <is>
+          <t>09:15p</t>
+        </is>
+      </c>
+      <c r="J43" s="4" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="K43" s="4" t="inlineStr">
+        <is>
+          <t>11:45a</t>
+        </is>
+      </c>
+      <c r="L43" s="4" t="inlineStr">
+        <is>
           <t>09:45p</t>
         </is>
       </c>
-      <c r="J43" s="4" t="n">
+      <c r="M43" s="4" t="n">
         <v>10</v>
-      </c>
-      <c r="K43" s="4" t="inlineStr">
-        <is>
-          <t>12:00p</t>
-        </is>
-      </c>
-      <c r="L43" s="4" t="inlineStr">
-        <is>
-          <t>09:30p</t>
-        </is>
-      </c>
-      <c r="M43" s="4" t="n">
-        <v>9.5</v>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
@@ -4816,51 +4816,51 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
+          <t>10:00a</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>02:00p</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
           <t>11:00a</t>
         </is>
       </c>
-      <c r="C44" s="4" t="inlineStr">
+      <c r="F44" s="4" t="inlineStr">
         <is>
           <t>09:00p</t>
         </is>
       </c>
-      <c r="D44" s="4" t="n">
+      <c r="G44" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="E44" s="4" t="inlineStr">
+      <c r="H44" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I44" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J44" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K44" s="4" t="inlineStr">
         <is>
           <t>10:00a</t>
         </is>
       </c>
-      <c r="F44" s="4" t="inlineStr">
-        <is>
-          <t>02:15p</t>
-        </is>
-      </c>
-      <c r="G44" s="4" t="n">
-        <v>4.25</v>
-      </c>
-      <c r="H44" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I44" s="4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="J44" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K44" s="4" t="inlineStr">
-        <is>
-          <t>10:15a</t>
-        </is>
-      </c>
       <c r="L44" s="4" t="inlineStr">
         <is>
-          <t>02:15p</t>
+          <t>02:00p</t>
         </is>
       </c>
       <c r="M44" s="4" t="n">
@@ -5148,25 +5148,25 @@
         </is>
       </c>
       <c r="B54" s="5" t="n">
-        <v>107.5</v>
+        <v>106</v>
       </c>
       <c r="E54" s="5" t="n">
-        <v>104.25</v>
+        <v>105.25</v>
       </c>
       <c r="H54" s="5" t="n">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="K54" s="5" t="n">
         <v>107</v>
       </c>
       <c r="N54" s="5" t="n">
-        <v>121.5</v>
+        <v>122.25</v>
       </c>
       <c r="Q54" s="5" t="n">
-        <v>105.25</v>
+        <v>106.25</v>
       </c>
       <c r="T54" s="5" t="n">
-        <v>109</v>
+        <v>108.75</v>
       </c>
       <c r="W54" s="5">
         <f>SUM(B54:T54)</f>
@@ -5328,7 +5328,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>+9.0</t>
+          <t>+7.5</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -5347,10 +5347,10 @@
         <v>8</v>
       </c>
       <c r="H60" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I60" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J60" t="n">
         <v>8</v>
@@ -5370,7 +5370,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>+8.8</t>
+          <t>+9.8</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -5389,19 +5389,19 @@
         <v>8</v>
       </c>
       <c r="H61" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I61" t="n">
+        <v>6</v>
+      </c>
+      <c r="J61" t="n">
+        <v>9</v>
+      </c>
+      <c r="K61" t="n">
+        <v>8</v>
+      </c>
+      <c r="L61" t="n">
         <v>5</v>
-      </c>
-      <c r="J61" t="n">
-        <v>8</v>
-      </c>
-      <c r="K61" t="n">
-        <v>7</v>
-      </c>
-      <c r="L61" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="62">
@@ -5412,7 +5412,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>-2.0</t>
+          <t>-3.0</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -5440,10 +5440,10 @@
         <v>8</v>
       </c>
       <c r="K62" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L62" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="63">
@@ -5479,7 +5479,7 @@
         <v>5</v>
       </c>
       <c r="J63" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K63" t="n">
         <v>6</v>
@@ -5496,7 +5496,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>+8.5</t>
+          <t>+9.2</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -5538,7 +5538,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>-2.8</t>
+          <t>-1.8</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -5566,7 +5566,7 @@
         <v>8</v>
       </c>
       <c r="K65" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L65" t="n">
         <v>6</v>
@@ -5580,7 +5580,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>+5.5</t>
+          <t>+5.2</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -5593,13 +5593,13 @@
         <v>12</v>
       </c>
       <c r="F66" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G66" t="n">
         <v>11</v>
       </c>
       <c r="H66" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I66" t="n">
         <v>6</v>
@@ -5611,7 +5611,7 @@
         <v>7</v>
       </c>
       <c r="L66" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="67">

</xml_diff>